<commit_message>
Draft CO2 manuscript package and SftO2 label fix
</commit_message>
<xml_diff>
--- a/results/supplemental_etables/Supplemental_eTables3_5_CO2_rSO2.xlsx
+++ b/results/supplemental_etables/Supplemental_eTables3_5_CO2_rSO2.xlsx
@@ -488,6 +488,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="24" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -506,7 +507,7 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Frontal SctO2 cohort</t>
+          <t>SftO2 cohort</t>
         </is>
       </c>
     </row>
@@ -1170,6 +1171,7 @@
         </is>
       </c>
     </row>
+    <row r="34"/>
     <row r="35">
       <c r="A35" s="8" t="inlineStr">
         <is>
@@ -1224,6 +1226,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="24" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -1242,7 +1245,7 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Frontal SctO2 cohort</t>
+          <t>SftO2 cohort</t>
         </is>
       </c>
     </row>
@@ -2588,6 +2591,7 @@
         </is>
       </c>
     </row>
+    <row r="65"/>
     <row r="66">
       <c r="A66" s="8" t="inlineStr">
         <is>
@@ -2640,13 +2644,13 @@
   </sheetData>
   <mergeCells count="8">
     <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A70:D70"/>
+    <mergeCell ref="A67:D67"/>
+    <mergeCell ref="A69:D69"/>
+    <mergeCell ref="A72:D72"/>
+    <mergeCell ref="A71:D71"/>
+    <mergeCell ref="A68:D68"/>
     <mergeCell ref="A66:D66"/>
-    <mergeCell ref="A67:D67"/>
-    <mergeCell ref="A68:D68"/>
-    <mergeCell ref="A69:D69"/>
-    <mergeCell ref="A70:D70"/>
-    <mergeCell ref="A71:D71"/>
-    <mergeCell ref="A72:D72"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2674,6 +2678,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="24" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -2692,7 +2697,7 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Frontal SctO2 cohort</t>
+          <t>SftO2 cohort</t>
         </is>
       </c>
     </row>
@@ -2850,6 +2855,7 @@
         </is>
       </c>
     </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>
@@ -2882,9 +2888,9 @@
   <mergeCells count="5">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A12:D12"/>
+    <mergeCell ref="A15:D15"/>
     <mergeCell ref="A13:D13"/>
     <mergeCell ref="A14:D14"/>
-    <mergeCell ref="A15:D15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Sync eTable 3-5 SftO2 labels
</commit_message>
<xml_diff>
--- a/results/supplemental_etables/Supplemental_eTables3_5_CO2_rSO2.xlsx
+++ b/results/supplemental_etables/Supplemental_eTables3_5_CO2_rSO2.xlsx
@@ -484,11 +484,10 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>eTable 3. Summary of timestamp-level outlier exclusions in left cerebral, right cerebral, and frontal cerebral tissue oxygen saturation cohorts</t>
-        </is>
-      </c>
-    </row>
-    <row r="2"/>
+          <t>eTable 3. Summary of timestamp-level outlier exclusions in left cerebral, right cerebral, and forearm tissue oxygen saturation cohorts</t>
+        </is>
+      </c>
+    </row>
     <row r="3" ht="24" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -1171,7 +1170,6 @@
         </is>
       </c>
     </row>
-    <row r="34"/>
     <row r="35">
       <c r="A35" s="8" t="inlineStr">
         <is>
@@ -1222,11 +1220,10 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>eTable 4. Missingness and imputation of intraoperative time-varying covariates in left cerebral, right cerebral, and frontal cerebral tissue oxygenation cohorts</t>
-        </is>
-      </c>
-    </row>
-    <row r="2"/>
+          <t>eTable 4. Missingness and imputation of intraoperative time-varying covariates in left cerebral, right cerebral, and forearm tissue oxygenation cohorts</t>
+        </is>
+      </c>
+    </row>
     <row r="3" ht="24" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -2591,7 +2588,6 @@
         </is>
       </c>
     </row>
-    <row r="65"/>
     <row r="66">
       <c r="A66" s="8" t="inlineStr">
         <is>
@@ -2674,11 +2670,10 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>eTable 5. Patient-level summary of intraoperative EtCO2 and tissue oxygenation in left cerebral, right cerebral, and frontal cerebral tissue oxygenation cohorts</t>
-        </is>
-      </c>
-    </row>
-    <row r="2"/>
+          <t>eTable 5. Patient-level summary of intraoperative EtCO2 and tissue oxygenation in left cerebral, right cerebral, and forearm tissue oxygenation cohorts</t>
+        </is>
+      </c>
+    </row>
     <row r="3" ht="24" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -2855,7 +2850,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>

</xml_diff>